<commit_message>
working ratio calculations, building vaccine priced search
</commit_message>
<xml_diff>
--- a/Heuristic/data/production_capacity_scenarios.xlsx
+++ b/Heuristic/data/production_capacity_scenarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/Heuristic/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{6259234B-0F6C-41FA-846B-135095B5B389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E243724-40D6-4E5E-83F5-BA2AA533A408}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{6259234B-0F6C-41FA-846B-135095B5B389}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDC56E01-CAF7-4BCF-8905-0C0C46C532B9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="base_capacity" sheetId="1" r:id="rId1"/>
@@ -446,6 +446,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">

</xml_diff>